<commit_message>
Network Audit complete for RLS & PSI
</commit_message>
<xml_diff>
--- a/data/BOM_Categories_Nokia.xlsx
+++ b/data/BOM_Categories_Nokia.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ZackerySimino\Downloads\LAMIS\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5B4D573-406C-4AB0-87AC-FB6255D063CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{986E4FBC-A805-43C6-A82A-268A9EEB6424}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="31380" yWindow="3150" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overrides" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="155">
   <si>
     <t>Part Number</t>
   </si>
@@ -438,13 +438,73 @@
   </si>
   <si>
     <t>Third Party Pluggable</t>
+  </si>
+  <si>
+    <t>3AL82040AB</t>
+  </si>
+  <si>
+    <t>SFP OSC FE/STM-1 ULH 1516NM 120KM -5/85</t>
+  </si>
+  <si>
+    <t>3KC48980AB</t>
+  </si>
+  <si>
+    <t>3KC49302AA</t>
+  </si>
+  <si>
+    <t>8EC3 -EQUIPT CONTROLLER PSS8 TEMP-HARDEN</t>
+  </si>
+  <si>
+    <t>EILAL EQUALIZED IN-LINE AMPLIFIER L-BAND</t>
+  </si>
+  <si>
+    <t>EILA EQUALIZED IN-LINE AMPLIFIER</t>
+  </si>
+  <si>
+    <t>3KC70175AA</t>
+  </si>
+  <si>
+    <t>3KC70424AA</t>
+  </si>
+  <si>
+    <t>16DC65-DC PWRFLTR(63A) PSS16II W SMPLTMG</t>
+  </si>
+  <si>
+    <t>RA5PB WB RAMAN AMP 5 PUMPS W/ BACK REF</t>
+  </si>
+  <si>
+    <t>3KC70525AA</t>
+  </si>
+  <si>
+    <t>8DG63029AB</t>
+  </si>
+  <si>
+    <t>3KC49010AA</t>
+  </si>
+  <si>
+    <t>32EC3 - HP EQUIPMENT CONTROLLER</t>
+  </si>
+  <si>
+    <t>3KC48990AB</t>
+  </si>
+  <si>
+    <t>16FAN2 - FAN UNIT - PSS16II</t>
+  </si>
+  <si>
+    <t>16UP2 - USER PANEL PSS16II</t>
+  </si>
+  <si>
+    <t>3KC48960AB</t>
+  </si>
+  <si>
+    <t>PSS16II-PSS16II SHELF (SHELF CHASSIS AND</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -470,6 +530,13 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -485,7 +552,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -551,11 +618,66 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF888888"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF888888"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF888888"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF888888"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF888888"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF888888"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF888888"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -600,9 +722,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 166" xfId="1" xr:uid="{39F79AC3-DBE1-4C37-9BFC-33DC5ADA9B1C}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -902,7 +1039,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C70"/>
+  <dimension ref="A1:C82"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.28515625" customWidth="1"/>
@@ -999,684 +1136,816 @@
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>18</v>
+      <c r="A9" s="16" t="s">
+        <v>150</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>21</v>
+        <v>4</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="16" t="s">
+        <v>137</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>23</v>
+        <v>4</v>
+      </c>
+      <c r="C10" s="19" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="13" t="s">
+        <v>137</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>24</v>
+        <v>152</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>26</v>
+        <v>153</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" s="21" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="3" t="s">
-        <v>28</v>
+      <c r="C13" s="20" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>19</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>19</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>19</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>19</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>19</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>19</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>19</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>19</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>19</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>19</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>19</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>19</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C26" s="3" t="s">
+      <c r="B30" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C30" s="3" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="4" t="s">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="13" t="s">
+        <v>148</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" s="13" t="s">
+        <v>146</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" s="13" t="s">
+        <v>147</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B27" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C27" s="5" t="s">
+      <c r="B37" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C37" s="5" t="s">
         <v>56</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="B28" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="C28" s="6" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" s="13" t="s">
-        <v>133</v>
-      </c>
-      <c r="B29" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" s="13" t="s">
-        <v>131</v>
-      </c>
-      <c r="B30" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="B31" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="C31" s="6" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="B32" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C32" s="6" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="B33" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C33" s="6" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="B34" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C34" s="6" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="B35" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C35" s="6" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="B36" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C36" s="6" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="B37" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C37" s="6" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="9" t="s">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>78</v>
+        <v>19</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" s="9" t="s">
-        <v>76</v>
+      <c r="A39" s="13" t="s">
+        <v>135</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C39" s="6" t="s">
-        <v>77</v>
+        <v>61</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="13" t="s">
-        <v>79</v>
+        <v>137</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>78</v>
+        <v>61</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>80</v>
+        <v>136</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="13" t="s">
-        <v>81</v>
+        <v>133</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>78</v>
+        <v>61</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>82</v>
+        <v>134</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="13" t="s">
+        <v>131</v>
+      </c>
+      <c r="B42" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="B43" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="B44" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="B45" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C45" s="6" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="B46" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C46" s="6" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="B47" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="B48" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="B49" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C49" s="6" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B50" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="B51" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C51" s="6" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="B52" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="B53" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="B42" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C42" s="3" t="s">
+      <c r="B54" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C54" s="3" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A43" s="13" t="s">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="B43" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C43" s="3" t="s">
+      <c r="B55" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C55" s="3" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A44" s="13" t="s">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="B44" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C44" s="3" t="s">
+      <c r="B56" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C56" s="3" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A45" s="13" t="s">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="B45" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C45" s="3" t="s">
+      <c r="B57" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C57" s="3" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A46" s="13" t="s">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A58" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="B46" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C46" s="3" t="s">
+      <c r="B58" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C58" s="3" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A47" s="13" t="s">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A59" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="B47" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C47" s="3" t="s">
+      <c r="B59" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C59" s="3" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A48" s="13" t="s">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60" s="13" t="s">
         <v>95</v>
       </c>
-      <c r="B48" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C48" s="3" t="s">
+      <c r="B60" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C60" s="3" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A49" s="13" t="s">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A61" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="B49" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C49" s="3" t="s">
+      <c r="B61" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C61" s="3" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A50" s="13" t="s">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A62" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="B50" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C50" s="3" t="s">
+      <c r="B62" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C62" s="3" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A51" s="13" t="s">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A63" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="B51" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C51" s="3" t="s">
+      <c r="B63" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C63" s="3" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A52" s="8" t="s">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A64" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="B52" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C52" s="11" t="s">
+      <c r="B64" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C64" s="11" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A53" s="8" t="s">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A65" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="B53" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C53" s="11" t="s">
+      <c r="B65" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C65" s="11" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A54" s="8" t="s">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A66" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="B54" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C54" s="11" t="s">
+      <c r="B66" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C66" s="11" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A55" s="8" t="s">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A67" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="B55" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C55" s="11" t="s">
+      <c r="B67" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C67" s="11" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A56" s="8" t="s">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A68" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="B56" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C56" s="11" t="s">
+      <c r="B68" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C68" s="11" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A57" s="8" t="s">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A69" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="B57" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C57" s="11" t="s">
+      <c r="B69" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C69" s="11" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A58" s="8" t="s">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A70" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="B58" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C58" s="11" t="s">
+      <c r="B70" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C70" s="11" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A59" s="10" t="s">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A71" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="B59" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C59" s="12" t="s">
+      <c r="B71" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C71" s="12" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A60" s="9" t="s">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A72" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="B60" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C60" s="14" t="s">
+      <c r="B72" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C72" s="14" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A61" s="9" t="s">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A73" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="B61" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C61" s="15" t="s">
+      <c r="B73" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C73" s="15" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A62" s="9" t="s">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A74" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="B62" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C62" s="14" t="s">
+      <c r="B74" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C74" s="14" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A63" s="9" t="s">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A75" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="B63" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C63" s="14" t="s">
+      <c r="B75" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C75" s="14" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A64" s="9" t="s">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A76" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="B64" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C64" s="14" t="s">
+      <c r="B76" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C76" s="14" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A65" s="9" t="s">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A77" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="B65" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C65" s="14" t="s">
+      <c r="B77" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C77" s="14" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A66" s="9" t="s">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A78" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="B66" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C66" s="14" t="s">
+      <c r="B78" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C78" s="14" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A67" s="9" t="s">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A79" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="B67" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C67" s="14" t="s">
+      <c r="B79" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C79" s="14" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A68" s="13" t="s">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A80" s="13" t="s">
         <v>127</v>
       </c>
-      <c r="B68" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C68" s="3" t="s">
+      <c r="B80" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C80" s="3" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A69" s="13" t="s">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A81" s="13" t="s">
         <v>129</v>
       </c>
-      <c r="B69" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C69" s="3" t="s">
+      <c r="B81" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C81" s="3" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A70" s="13" t="s">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A82" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="B70" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C70" s="3" t="s">
+      <c r="B82" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C82" s="3" t="s">
         <v>58</v>
       </c>
     </row>

</xml_diff>